<commit_message>
Update at 14:03 on 07/27/2020
</commit_message>
<xml_diff>
--- a/site_libs/fall 2020.xlsx
+++ b/site_libs/fall 2020.xlsx
@@ -1,20 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23001"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Portfolio\site_libs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB4EB6CB-43A5-4CC7-8A1A-80231397519D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Schedule" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="WDD Schedule" sheetId="2" r:id="rId5"/>
-    <sheet state="visible" name="TA" sheetId="3" r:id="rId6"/>
-    <sheet state="hidden" name="Copy of Fall 2020" sheetId="4" r:id="rId7"/>
+    <sheet name="Schedule" sheetId="1" r:id="rId1"/>
+    <sheet name="WDD Schedule" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet name="TA" sheetId="3" r:id="rId3"/>
+    <sheet name="Copy of Fall 2020" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="123">
   <si>
     <t>Monday</t>
   </si>
@@ -396,62 +415,87 @@
 Machine Learning
 Falin</t>
   </si>
+  <si>
+    <t>121b</t>
+  </si>
+  <si>
+    <t>JavaScript</t>
+  </si>
+  <si>
+    <t>10:15-11:15</t>
+  </si>
+  <si>
+    <t>Barney</t>
+  </si>
+  <si>
+    <t>CSE 121b JavaScript Barney Remote</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="h:mm:ss am/pm"/>
-  </numFmts>
-  <fonts count="11">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
-    <font/>
     <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF999999"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF0076B6"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF020202"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF0076B6"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF020202"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -459,7 +503,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -475,119 +519,121 @@
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="34">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="19" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="19" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="top"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment readingOrder="0" vertical="top"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="top"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="top"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="top"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -777,51 +823,59 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
+  <dimension ref="A1:U36"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="11.71"/>
-    <col customWidth="1" min="2" max="2" width="14.43"/>
-    <col customWidth="1" min="3" max="3" width="8.71"/>
-    <col customWidth="1" min="4" max="4" width="14.29"/>
-    <col customWidth="1" min="5" max="5" width="8.71"/>
-    <col customWidth="1" min="7" max="7" width="9.86"/>
-    <col customWidth="1" min="8" max="8" width="14.43"/>
-    <col customWidth="1" min="9" max="9" width="9.86"/>
-    <col customWidth="1" min="12" max="12" width="6.0"/>
-    <col customWidth="1" min="13" max="13" width="10.86"/>
-    <col customWidth="1" min="14" max="14" width="5.57"/>
-    <col customWidth="1" min="15" max="15" width="16.14"/>
-    <col customWidth="1" min="16" max="17" width="7.71"/>
-    <col customWidth="1" min="18" max="18" width="5.57"/>
-    <col customWidth="1" min="19" max="19" width="11.0"/>
-    <col customWidth="1" min="20" max="20" width="9.86"/>
-    <col customWidth="1" min="21" max="21" width="5.0"/>
+    <col min="1" max="1" width="11.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" customWidth="1"/>
+    <col min="4" max="4" width="10.42578125" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" customWidth="1"/>
+    <col min="8" max="8" width="10.140625" customWidth="1"/>
+    <col min="9" max="9" width="9.85546875" customWidth="1"/>
+    <col min="12" max="12" width="6" customWidth="1"/>
+    <col min="13" max="13" width="10.85546875" customWidth="1"/>
+    <col min="14" max="14" width="5.5703125" customWidth="1"/>
+    <col min="15" max="15" width="16.140625" customWidth="1"/>
+    <col min="16" max="17" width="7.7109375" customWidth="1"/>
+    <col min="18" max="18" width="5.5703125" customWidth="1"/>
+    <col min="19" max="19" width="11" customWidth="1"/>
+    <col min="20" max="20" width="9.85546875" customWidth="1"/>
+    <col min="21" max="21" width="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="B1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="C1" s="26"/>
+      <c r="D1" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="E1" s="26"/>
+      <c r="F1" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="G1" s="26"/>
+      <c r="H1" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="I1" s="26"/>
+      <c r="J1" s="25" t="s">
         <v>4</v>
       </c>
+      <c r="K1" s="26"/>
       <c r="L1" s="1"/>
       <c r="M1" s="2" t="s">
         <v>5</v>
@@ -851,60 +905,62 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
-        <v>0.3229166666666667</v>
+        <v>0.32291666666666669</v>
       </c>
       <c r="B2" s="4"/>
-      <c r="D2" s="5"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="6"/>
       <c r="E2" s="6"/>
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
-      <c r="H2" s="5"/>
+      <c r="H2" s="6"/>
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
       <c r="L2" s="4"/>
-      <c r="M2" s="7" t="s">
+      <c r="M2" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="N2" s="7">
-        <v>450.0</v>
-      </c>
-      <c r="O2" s="7" t="s">
-        <v>15</v>
+      <c r="N2" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="O2" s="13" t="s">
+        <v>119</v>
       </c>
       <c r="P2" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q2" s="7">
-        <v>347.0</v>
-      </c>
-      <c r="R2" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="S2" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="T2" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="U2" s="7">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>23</v>
+      </c>
+      <c r="Q2" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="R2" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="S2" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="T2" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="U2" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A3" s="8">
-        <v>0.3333333333333333</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="B3" s="4"/>
-      <c r="D3" s="5" t="s">
+      <c r="C3" s="31"/>
+      <c r="D3" s="27" t="s">
         <v>20</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
-      <c r="H3" s="5" t="str">
+      <c r="H3" s="27" t="str">
         <f>D3</f>
         <v>MATH 488
 Consulting
@@ -916,41 +972,44 @@
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
       <c r="M3" s="7" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="N3" s="7">
-        <v>325.0</v>
+        <v>450</v>
       </c>
       <c r="O3" s="7" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="P3" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q3" s="7" t="s">
-        <v>24</v>
+        <v>16</v>
+      </c>
+      <c r="Q3" s="7">
+        <v>347</v>
       </c>
       <c r="R3" s="7" t="s">
         <v>17</v>
       </c>
       <c r="S3" s="7" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="T3" s="7" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="U3" s="7">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4" s="8">
         <v>0.34375</v>
       </c>
       <c r="B4" s="4"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="32"/>
       <c r="E4" s="6"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
+      <c r="H4" s="32"/>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -959,90 +1018,131 @@
         <v>21</v>
       </c>
       <c r="N4" s="7">
-        <v>488.0</v>
+        <v>325</v>
       </c>
       <c r="O4" s="7" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="P4" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q4" s="7">
-        <v>229.0</v>
+        <v>23</v>
+      </c>
+      <c r="Q4" s="7" t="s">
+        <v>24</v>
       </c>
       <c r="R4" s="7" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="S4" s="7" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="T4" s="7" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="U4" s="7">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5" s="8">
-        <v>0.3541666666666667</v>
+        <v>0.35416666666666669</v>
       </c>
       <c r="B5" s="4"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="32"/>
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
+      <c r="H5" s="32"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
-    </row>
-    <row r="6">
+      <c r="M5" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="N5" s="7">
+        <v>488</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="P5" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q5" s="7">
+        <v>229</v>
+      </c>
+      <c r="R5" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="S5" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="T5" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="U5" s="7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A6" s="8">
-        <v>0.3645833333333333</v>
+        <v>0.36458333333333331</v>
       </c>
       <c r="B6" s="4"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="32"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
+      <c r="H6" s="32"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
-    </row>
-    <row r="7">
+      <c r="U6">
+        <f>SUM(U2:U5)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A7" s="8">
         <v>0.375</v>
       </c>
       <c r="B7" s="4"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="32"/>
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
+      <c r="H7" s="32"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
       <c r="L7" s="4"/>
     </row>
-    <row r="8">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A8" s="8">
-        <v>0.3854166666666667</v>
+        <v>0.38541666666666669</v>
       </c>
       <c r="B8" s="4"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="32"/>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
+      <c r="H8" s="32"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
-      <c r="M8" s="9" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="9">
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A9" s="8">
-        <v>0.3958333333333333</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="B9" s="4"/>
+      <c r="C9" s="31"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
@@ -1052,15 +1152,16 @@
       <c r="J9" s="4"/>
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
-      <c r="M9" s="10" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="10">
+      <c r="M9" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A10" s="8">
         <v>0.40625</v>
       </c>
       <c r="B10" s="4"/>
+      <c r="C10" s="31"/>
       <c r="D10" s="11"/>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
@@ -1070,12 +1171,16 @@
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
-    </row>
-    <row r="11">
+      <c r="M10" s="10" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A11" s="8">
-        <v>0.4166666666666667</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="B11" s="4"/>
+      <c r="C11" s="31"/>
       <c r="D11" s="11"/>
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
@@ -1086,68 +1191,80 @@
       <c r="K11" s="4"/>
       <c r="L11" s="4"/>
     </row>
-    <row r="12">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A12" s="8">
-        <v>0.4270833333333333</v>
-      </c>
-      <c r="B12" s="1"/>
-      <c r="C12" s="12" t="s">
+        <v>0.42708333333333331</v>
+      </c>
+      <c r="B12" s="4"/>
+      <c r="C12" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="11"/>
+      <c r="D12" s="33" t="s">
+        <v>122</v>
+      </c>
       <c r="E12" s="4"/>
-      <c r="F12" s="1" t="str">
-        <f>B12</f>
-        <v/>
-      </c>
-      <c r="G12" s="12" t="s">
+      <c r="F12" s="4"/>
+      <c r="G12" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="H12" s="11"/>
+      <c r="H12" s="33" t="s">
+        <v>122</v>
+      </c>
       <c r="I12" s="4"/>
-      <c r="J12" s="1"/>
-    </row>
-    <row r="13">
+      <c r="J12" s="4"/>
+      <c r="K12" s="31"/>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A13" s="8">
         <v>0.4375</v>
       </c>
-      <c r="B13" s="1"/>
-      <c r="D13" s="11"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="32"/>
+      <c r="D13" s="33"/>
       <c r="E13" s="4"/>
-      <c r="F13" s="1"/>
-      <c r="H13" s="11"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="32"/>
+      <c r="H13" s="33"/>
       <c r="I13" s="4"/>
-      <c r="J13" s="1"/>
-    </row>
-    <row r="14">
+      <c r="J13" s="4"/>
+      <c r="K13" s="31"/>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A14" s="8">
-        <v>0.4479166666666667</v>
-      </c>
-      <c r="B14" s="1"/>
-      <c r="D14" s="11"/>
+        <v>0.44791666666666669</v>
+      </c>
+      <c r="B14" s="4"/>
+      <c r="C14" s="32"/>
+      <c r="D14" s="33"/>
       <c r="E14" s="4"/>
-      <c r="F14" s="1"/>
-      <c r="H14" s="11"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="32"/>
+      <c r="H14" s="33"/>
       <c r="I14" s="4"/>
-      <c r="J14" s="1"/>
-    </row>
-    <row r="15">
+      <c r="J14" s="4"/>
+      <c r="K14" s="31"/>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A15" s="8">
-        <v>0.4583333333333333</v>
-      </c>
-      <c r="B15" s="1"/>
-      <c r="D15" s="11"/>
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="B15" s="4"/>
+      <c r="C15" s="32"/>
+      <c r="D15" s="33"/>
       <c r="E15" s="4"/>
-      <c r="F15" s="1"/>
-      <c r="H15" s="11"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="32"/>
+      <c r="H15" s="33"/>
       <c r="I15" s="4"/>
-      <c r="J15" s="1"/>
-    </row>
-    <row r="16">
+      <c r="J15" s="4"/>
+      <c r="K15" s="31"/>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A16" s="8">
         <v>0.46875</v>
       </c>
       <c r="B16" s="4"/>
+      <c r="C16" s="31"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
@@ -1155,69 +1272,88 @@
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
       <c r="J16" s="4"/>
-    </row>
-    <row r="17">
+      <c r="K16" s="31"/>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="8">
-        <v>0.4791666666666667</v>
-      </c>
-      <c r="B17" s="5" t="s">
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="B17" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="F17" s="5" t="str">
+      <c r="C17" s="31"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="27" t="str">
         <f>B17</f>
         <v>CSE 450
 Machine Learning
 Burton 
 STC  394</v>
       </c>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="13"/>
-      <c r="J17" s="5" t="str">
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="27" t="str">
         <f>F17</f>
         <v>CSE 450
 Machine Learning
 Burton 
 STC  394</v>
       </c>
-    </row>
-    <row r="18">
+      <c r="K17" s="31"/>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="8">
-        <v>0.4895833333333333</v>
-      </c>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="13"/>
-    </row>
-    <row r="19">
+        <v>0.48958333333333331</v>
+      </c>
+      <c r="B18" s="32"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="32"/>
+      <c r="K18" s="31"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="8">
         <v>0.5</v>
       </c>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="G19" s="13"/>
-      <c r="H19" s="13"/>
-      <c r="I19" s="13"/>
-    </row>
-    <row r="20">
+      <c r="B19" s="32"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="32"/>
+      <c r="K19" s="31"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="8">
-        <v>0.5104166666666666</v>
-      </c>
+        <v>0.51041666666666663</v>
+      </c>
+      <c r="B20" s="32"/>
+      <c r="C20" s="31"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
+      <c r="F20" s="32"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
-    </row>
-    <row r="21">
+      <c r="J20" s="32"/>
+      <c r="K20" s="31"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="8">
-        <v>0.5208333333333334</v>
+        <v>0.52083333333333337</v>
       </c>
       <c r="B21" s="4"/>
+      <c r="C21" s="31"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
@@ -1225,186 +1361,245 @@
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
       <c r="J21" s="4"/>
-    </row>
-    <row r="22">
+      <c r="K21" s="31"/>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="8">
         <v>0.53125</v>
       </c>
       <c r="B22" s="4"/>
+      <c r="C22" s="31"/>
       <c r="D22" s="4"/>
-      <c r="E22" s="12" t="s">
+      <c r="E22" s="29" t="s">
         <v>34</v>
       </c>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
-      <c r="I22" s="12" t="s">
+      <c r="I22" s="29" t="s">
         <v>35</v>
       </c>
       <c r="J22" s="4"/>
-    </row>
-    <row r="23">
+      <c r="K22" s="31"/>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="8">
-        <v>0.5416666666666666</v>
+        <v>0.54166666666666663</v>
       </c>
       <c r="B23" s="4"/>
+      <c r="C23" s="31"/>
       <c r="D23" s="4"/>
+      <c r="E23" s="32"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
+      <c r="I23" s="32"/>
       <c r="J23" s="4"/>
-    </row>
-    <row r="24">
+      <c r="K23" s="31"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="8">
-        <v>0.5520833333333334</v>
+        <v>0.55208333333333337</v>
       </c>
       <c r="B24" s="4"/>
+      <c r="C24" s="31"/>
       <c r="D24" s="4"/>
+      <c r="E24" s="32"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
+      <c r="I24" s="32"/>
       <c r="J24" s="4"/>
-    </row>
-    <row r="25">
+      <c r="K24" s="31"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" s="8">
         <v>0.5625</v>
       </c>
       <c r="B25" s="4"/>
+      <c r="C25" s="31"/>
       <c r="D25" s="4"/>
+      <c r="E25" s="32"/>
       <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
+      <c r="I25" s="32"/>
       <c r="J25" s="4"/>
-    </row>
-    <row r="26">
+      <c r="K25" s="31"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="8">
-        <v>0.5729166666666666</v>
-      </c>
-    </row>
-    <row r="27">
+        <v>0.57291666666666663</v>
+      </c>
+      <c r="B26" s="31"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
+      <c r="E26" s="31"/>
+      <c r="F26" s="31"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="31"/>
+      <c r="J26" s="31"/>
+      <c r="K26" s="31"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" s="8">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="B27" s="1" t="s">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="B27" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D27" s="1"/>
-      <c r="E27" s="14" t="s">
+      <c r="C27" s="31"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="F27" s="1" t="str">
+      <c r="F27" s="25" t="str">
         <f>B27</f>
         <v>MATH 325
 Intermediate Stats 
 Saunders 
 Remote</v>
       </c>
-      <c r="H27" s="1"/>
-      <c r="I27" s="14" t="s">
+      <c r="G27" s="31"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="J27" s="1" t="str">
+      <c r="J27" s="25" t="str">
         <f>F27</f>
         <v>MATH 325
 Intermediate Stats 
 Saunders 
 Remote</v>
       </c>
-    </row>
-    <row r="28">
+      <c r="K27" s="31"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="8">
         <v>0.59375</v>
       </c>
-      <c r="D28" s="1"/>
-      <c r="H28" s="1"/>
-    </row>
-    <row r="29">
+      <c r="B28" s="32"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="31"/>
+      <c r="H28" s="4"/>
+      <c r="I28" s="32"/>
+      <c r="J28" s="32"/>
+      <c r="K28" s="31"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" s="8">
-        <v>0.6041666666666666</v>
-      </c>
-      <c r="D29" s="1"/>
-      <c r="H29" s="1"/>
-    </row>
-    <row r="30">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="B29" s="32"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="32"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="31"/>
+      <c r="H29" s="4"/>
+      <c r="I29" s="32"/>
+      <c r="J29" s="32"/>
+      <c r="K29" s="31"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="8">
-        <v>0.6145833333333334</v>
-      </c>
-      <c r="D30" s="1"/>
-      <c r="H30" s="1"/>
-    </row>
-    <row r="31">
+        <v>0.61458333333333337</v>
+      </c>
+      <c r="B30" s="32"/>
+      <c r="C30" s="31"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="32"/>
+      <c r="F30" s="32"/>
+      <c r="G30" s="31"/>
+      <c r="H30" s="4"/>
+      <c r="I30" s="32"/>
+      <c r="J30" s="32"/>
+      <c r="K30" s="31"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" s="8">
         <v>0.625</v>
       </c>
       <c r="B31" s="4"/>
+      <c r="C31" s="31"/>
       <c r="D31" s="4"/>
       <c r="E31" s="4"/>
-      <c r="F31" s="1" t="s">
+      <c r="F31" s="4" t="s">
         <v>39</v>
       </c>
+      <c r="G31" s="31"/>
       <c r="H31" s="4"/>
       <c r="I31" s="4"/>
       <c r="J31" s="4"/>
-    </row>
-    <row r="32">
+      <c r="K31" s="31"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" s="8">
-        <v>0.6354166666666666</v>
-      </c>
-      <c r="B32" s="5"/>
-      <c r="C32" s="5"/>
-      <c r="D32" s="5"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="5"/>
-      <c r="G32" s="5"/>
-      <c r="H32" s="5"/>
-      <c r="I32" s="5"/>
-      <c r="J32" s="5"/>
-    </row>
-    <row r="33">
+        <v>0.63541666666666663</v>
+      </c>
+      <c r="B32" s="6"/>
+      <c r="C32" s="6"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="6"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="6"/>
+      <c r="H32" s="6"/>
+      <c r="I32" s="6"/>
+      <c r="J32" s="6"/>
+      <c r="K32" s="31"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" s="8">
-        <v>0.6458333333333334</v>
-      </c>
-      <c r="B33" s="5"/>
-      <c r="C33" s="5"/>
-      <c r="D33" s="5"/>
-      <c r="E33" s="5"/>
-      <c r="F33" s="5"/>
-      <c r="G33" s="5"/>
-      <c r="H33" s="5"/>
-      <c r="I33" s="5"/>
-      <c r="J33" s="5"/>
-    </row>
-    <row r="34">
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="B33" s="6"/>
+      <c r="C33" s="6"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="6"/>
+      <c r="H33" s="6"/>
+      <c r="I33" s="6"/>
+      <c r="J33" s="6"/>
+      <c r="K33" s="31"/>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" s="8">
         <v>0.65625</v>
       </c>
-      <c r="B34" s="5"/>
-      <c r="C34" s="5"/>
-      <c r="D34" s="5"/>
-      <c r="E34" s="5"/>
-      <c r="F34" s="5"/>
-      <c r="G34" s="5"/>
-      <c r="H34" s="5"/>
-      <c r="I34" s="5"/>
-      <c r="J34" s="5"/>
-    </row>
-    <row r="35">
+      <c r="B34" s="6"/>
+      <c r="C34" s="6"/>
+      <c r="D34" s="6"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="6"/>
+      <c r="G34" s="6"/>
+      <c r="H34" s="6"/>
+      <c r="I34" s="6"/>
+      <c r="J34" s="6"/>
+      <c r="K34" s="31"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" s="8">
-        <v>0.6666666666666666</v>
-      </c>
-      <c r="B35" s="5"/>
-      <c r="C35" s="5"/>
-      <c r="D35" s="5"/>
-      <c r="E35" s="5"/>
-      <c r="F35" s="5"/>
-      <c r="G35" s="5"/>
-      <c r="H35" s="5"/>
-      <c r="I35" s="5"/>
-      <c r="J35" s="5"/>
-    </row>
-    <row r="36">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="B35" s="6"/>
+      <c r="C35" s="6"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="6"/>
+      <c r="G35" s="6"/>
+      <c r="H35" s="6"/>
+      <c r="I35" s="6"/>
+      <c r="J35" s="6"/>
+      <c r="K35" s="31"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" s="8">
-        <v>0.6770833333333334</v>
+        <v>0.67708333333333337</v>
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="4"/>
@@ -1415,75 +1610,84 @@
       <c r="H36" s="4"/>
       <c r="I36" s="4"/>
       <c r="J36" s="4"/>
+      <c r="K36" s="31"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="J1:K1"/>
+  <mergeCells count="21">
+    <mergeCell ref="B27:B30"/>
+    <mergeCell ref="F27:F30"/>
+    <mergeCell ref="J27:J30"/>
+    <mergeCell ref="D12:D15"/>
+    <mergeCell ref="H12:H15"/>
+    <mergeCell ref="C12:C15"/>
+    <mergeCell ref="G12:G15"/>
+    <mergeCell ref="B17:B20"/>
+    <mergeCell ref="F17:F20"/>
+    <mergeCell ref="J17:J20"/>
     <mergeCell ref="D3:D8"/>
     <mergeCell ref="H3:H8"/>
     <mergeCell ref="E22:E25"/>
     <mergeCell ref="E27:E30"/>
     <mergeCell ref="I22:I25"/>
     <mergeCell ref="I27:I30"/>
-    <mergeCell ref="C12:C15"/>
-    <mergeCell ref="G12:G15"/>
-    <mergeCell ref="B17:B20"/>
-    <mergeCell ref="F17:F20"/>
-    <mergeCell ref="J17:J20"/>
-    <mergeCell ref="B27:B30"/>
-    <mergeCell ref="F27:F30"/>
-    <mergeCell ref="J27:J30"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="J1:K1"/>
   </mergeCells>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
+  <dimension ref="A1:U35"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="11.71"/>
-    <col customWidth="1" min="2" max="2" width="14.43"/>
-    <col customWidth="1" min="3" max="3" width="8.71"/>
-    <col customWidth="1" min="4" max="4" width="14.29"/>
-    <col customWidth="1" min="5" max="5" width="8.71"/>
-    <col customWidth="1" min="7" max="7" width="9.86"/>
-    <col customWidth="1" min="8" max="8" width="14.43"/>
-    <col customWidth="1" min="9" max="9" width="9.86"/>
-    <col customWidth="1" min="12" max="12" width="6.0"/>
-    <col customWidth="1" min="13" max="13" width="10.86"/>
-    <col customWidth="1" min="14" max="14" width="5.57"/>
-    <col customWidth="1" min="15" max="15" width="16.14"/>
-    <col customWidth="1" min="16" max="17" width="7.71"/>
-    <col customWidth="1" min="18" max="18" width="5.57"/>
-    <col customWidth="1" min="19" max="19" width="11.0"/>
-    <col customWidth="1" min="20" max="20" width="9.86"/>
-    <col customWidth="1" min="21" max="21" width="5.0"/>
+    <col min="1" max="1" width="11.7109375" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" customWidth="1"/>
+    <col min="7" max="7" width="9.85546875" customWidth="1"/>
+    <col min="8" max="8" width="14.42578125" customWidth="1"/>
+    <col min="9" max="9" width="9.85546875" customWidth="1"/>
+    <col min="12" max="12" width="6" customWidth="1"/>
+    <col min="13" max="13" width="10.85546875" customWidth="1"/>
+    <col min="14" max="14" width="5.5703125" customWidth="1"/>
+    <col min="15" max="15" width="16.140625" customWidth="1"/>
+    <col min="16" max="17" width="7.7109375" customWidth="1"/>
+    <col min="18" max="18" width="5.5703125" customWidth="1"/>
+    <col min="19" max="19" width="11" customWidth="1"/>
+    <col min="20" max="20" width="9.85546875" customWidth="1"/>
+    <col min="21" max="21" width="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="B1" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="C1" s="26"/>
+      <c r="D1" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="E1" s="26"/>
+      <c r="F1" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="G1" s="26"/>
+      <c r="H1" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="I1" s="26"/>
+      <c r="J1" s="25" t="s">
         <v>4</v>
       </c>
+      <c r="K1" s="26"/>
       <c r="L1" s="1"/>
       <c r="M1" s="2" t="s">
         <v>5</v>
@@ -1513,18 +1717,18 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" s="8">
-        <v>0.3333333333333333</v>
+        <v>0.33333333333333331</v>
       </c>
       <c r="B2" s="4"/>
-      <c r="D2" s="11" t="s">
+      <c r="D2" s="30" t="s">
         <v>40</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
-      <c r="H2" s="11" t="str">
+      <c r="H2" s="30" t="str">
         <f>D2</f>
         <v>CSE 341
 Web Backend 2
@@ -1539,7 +1743,7 @@
         <v>14</v>
       </c>
       <c r="N2" s="2">
-        <v>450.0</v>
+        <v>450</v>
       </c>
       <c r="O2" s="2" t="s">
         <v>15</v>
@@ -1548,7 +1752,7 @@
         <v>16</v>
       </c>
       <c r="Q2" s="2">
-        <v>347.0</v>
+        <v>347</v>
       </c>
       <c r="R2" s="2" t="s">
         <v>17</v>
@@ -1560,17 +1764,19 @@
         <v>19</v>
       </c>
       <c r="U2" s="2">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A3" s="8">
         <v>0.34375</v>
       </c>
       <c r="B3" s="4"/>
+      <c r="D3" s="26"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
+      <c r="H3" s="26"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
@@ -1579,7 +1785,7 @@
         <v>21</v>
       </c>
       <c r="N3" s="2">
-        <v>325.0</v>
+        <v>325</v>
       </c>
       <c r="O3" s="2" t="s">
         <v>22</v>
@@ -1600,17 +1806,19 @@
         <v>26</v>
       </c>
       <c r="U3" s="2">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4" s="8">
-        <v>0.3541666666666667</v>
+        <v>0.35416666666666669</v>
       </c>
       <c r="B4" s="4"/>
+      <c r="D4" s="26"/>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
+      <c r="H4" s="26"/>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -1619,7 +1827,7 @@
         <v>41</v>
       </c>
       <c r="N4" s="2">
-        <v>330.0</v>
+        <v>330</v>
       </c>
       <c r="O4" s="2" t="s">
         <v>42</v>
@@ -1628,7 +1836,7 @@
         <v>16</v>
       </c>
       <c r="Q4" s="2">
-        <v>347.0</v>
+        <v>347</v>
       </c>
       <c r="R4" s="2" t="s">
         <v>29</v>
@@ -1636,21 +1844,23 @@
       <c r="S4" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="T4" s="15" t="s">
+      <c r="T4" s="13" t="s">
         <v>44</v>
       </c>
       <c r="U4" s="2">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5" s="8">
-        <v>0.3645833333333333</v>
+        <v>0.36458333333333331</v>
       </c>
       <c r="B5" s="4"/>
+      <c r="D5" s="26"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
+      <c r="H5" s="26"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -1659,7 +1869,7 @@
         <v>14</v>
       </c>
       <c r="N5" s="2">
-        <v>341.0</v>
+        <v>341</v>
       </c>
       <c r="O5" s="2" t="s">
         <v>45</v>
@@ -1676,34 +1886,38 @@
       <c r="S5" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="T5" s="15" t="s">
+      <c r="T5" s="13" t="s">
         <v>47</v>
       </c>
       <c r="U5" s="2">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A6" s="8">
         <v>0.375</v>
       </c>
       <c r="B6" s="4"/>
+      <c r="D6" s="26"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
+      <c r="H6" s="26"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
     </row>
-    <row r="7">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A7" s="8">
-        <v>0.3854166666666667</v>
+        <v>0.38541666666666669</v>
       </c>
       <c r="B7" s="4"/>
+      <c r="D7" s="26"/>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
+      <c r="H7" s="26"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -1712,9 +1926,9 @@
         <v>32</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A8" s="8">
-        <v>0.3958333333333333</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="B8" s="4"/>
       <c r="D8" s="4"/>
@@ -1730,18 +1944,18 @@
         <v>33</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A9" s="8">
         <v>0.40625</v>
       </c>
       <c r="B9" s="4"/>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="30" t="s">
         <v>48</v>
       </c>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
-      <c r="H9" s="11" t="s">
+      <c r="H9" s="30" t="s">
         <v>48</v>
       </c>
       <c r="I9" s="4"/>
@@ -1749,69 +1963,85 @@
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
     </row>
-    <row r="10">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A10" s="8">
-        <v>0.4166666666666667</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="B10" s="4"/>
+      <c r="D10" s="26"/>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
+      <c r="H10" s="26"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
     </row>
-    <row r="11">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A11" s="8">
-        <v>0.4270833333333333</v>
+        <v>0.42708333333333331</v>
       </c>
       <c r="B11" s="1"/>
-      <c r="C11" s="12" t="s">
+      <c r="C11" s="28" t="s">
         <v>34</v>
       </c>
+      <c r="D11" s="26"/>
       <c r="E11" s="4"/>
-      <c r="F11" s="1" t="str">
+      <c r="F11" s="1">
         <f>B11</f>
-        <v/>
-      </c>
-      <c r="G11" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="G11" s="28" t="s">
         <v>35</v>
       </c>
+      <c r="H11" s="26"/>
       <c r="I11" s="4"/>
       <c r="J11" s="1"/>
     </row>
-    <row r="12">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A12" s="8">
         <v>0.4375</v>
       </c>
       <c r="B12" s="1"/>
+      <c r="C12" s="26"/>
+      <c r="D12" s="26"/>
       <c r="E12" s="4"/>
       <c r="F12" s="1"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="26"/>
       <c r="I12" s="4"/>
       <c r="J12" s="1"/>
     </row>
-    <row r="13">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A13" s="8">
-        <v>0.4479166666666667</v>
+        <v>0.44791666666666669</v>
       </c>
       <c r="B13" s="1"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
       <c r="E13" s="4"/>
       <c r="F13" s="1"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
       <c r="I13" s="4"/>
       <c r="J13" s="1"/>
     </row>
-    <row r="14">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A14" s="8">
-        <v>0.4583333333333333</v>
+        <v>0.45833333333333331</v>
       </c>
       <c r="B14" s="1"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="26"/>
       <c r="E14" s="4"/>
       <c r="F14" s="1"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="26"/>
       <c r="I14" s="4"/>
       <c r="J14" s="1"/>
     </row>
-    <row r="15">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A15" s="8">
         <v>0.46875</v>
       </c>
@@ -1824,26 +2054,26 @@
       <c r="I15" s="4"/>
       <c r="J15" s="4"/>
     </row>
-    <row r="16">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A16" s="8">
-        <v>0.4791666666666667</v>
-      </c>
-      <c r="B16" s="5" t="s">
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="B16" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="5" t="str">
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="27" t="str">
         <f>B16</f>
         <v>CSE 450
 Machine Learning
 Burton 
 STC  394</v>
       </c>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="13"/>
-      <c r="J16" s="5" t="str">
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
+      <c r="J16" s="27" t="str">
         <f>F16</f>
         <v>CSE 450
 Machine Learning
@@ -1851,39 +2081,48 @@
 STC  394</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" s="8">
-        <v>0.4895833333333333</v>
-      </c>
-      <c r="D17" s="13"/>
-      <c r="E17" s="13"/>
-      <c r="G17" s="13"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="13"/>
-    </row>
-    <row r="18">
+        <v>0.48958333333333331</v>
+      </c>
+      <c r="B17" s="26"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="26"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="8">
         <v>0.5</v>
       </c>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="13"/>
-    </row>
-    <row r="19">
+      <c r="B18" s="26"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="26"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+      <c r="I18" s="12"/>
+      <c r="J18" s="26"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="8">
-        <v>0.5104166666666666</v>
-      </c>
+        <v>0.51041666666666663</v>
+      </c>
+      <c r="B19" s="26"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
+      <c r="F19" s="26"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
-    </row>
-    <row r="20">
+      <c r="J19" s="26"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="8">
-        <v>0.5208333333333334</v>
+        <v>0.52083333333333337</v>
       </c>
       <c r="B20" s="4"/>
       <c r="D20" s="4"/>
@@ -1894,73 +2133,79 @@
       <c r="I20" s="4"/>
       <c r="J20" s="4"/>
     </row>
-    <row r="21">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="8">
         <v>0.53125</v>
       </c>
       <c r="B21" s="4"/>
       <c r="D21" s="4"/>
-      <c r="E21" s="12" t="s">
+      <c r="E21" s="28" t="s">
         <v>34</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
-      <c r="I21" s="12" t="s">
+      <c r="I21" s="28" t="s">
         <v>35</v>
       </c>
       <c r="J21" s="4"/>
     </row>
-    <row r="22">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" s="8">
-        <v>0.5416666666666666</v>
+        <v>0.54166666666666663</v>
       </c>
       <c r="B22" s="4"/>
       <c r="D22" s="4"/>
+      <c r="E22" s="26"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
+      <c r="I22" s="26"/>
       <c r="J22" s="4"/>
     </row>
-    <row r="23">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" s="8">
-        <v>0.5520833333333334</v>
+        <v>0.55208333333333337</v>
       </c>
       <c r="B23" s="4"/>
       <c r="D23" s="4"/>
+      <c r="E23" s="26"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
+      <c r="I23" s="26"/>
       <c r="J23" s="4"/>
     </row>
-    <row r="24">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="8">
         <v>0.5625</v>
       </c>
       <c r="B24" s="4"/>
       <c r="D24" s="4"/>
+      <c r="E24" s="26"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
+      <c r="I24" s="26"/>
       <c r="J24" s="4"/>
     </row>
-    <row r="25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" s="8">
-        <v>0.5729166666666666</v>
-      </c>
-    </row>
-    <row r="26">
+        <v>0.57291666666666663</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" s="8">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="B26" s="1" t="s">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="B26" s="25" t="s">
         <v>37</v>
       </c>
       <c r="D26" s="1"/>
-      <c r="E26" s="14" t="s">
+      <c r="E26" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="F26" s="1" t="str">
+      <c r="F26" s="25" t="str">
         <f>B26</f>
         <v>MATH 325
 Intermediate Stats 
@@ -1968,10 +2213,10 @@
 Remote</v>
       </c>
       <c r="H26" s="1"/>
-      <c r="I26" s="14" t="s">
+      <c r="I26" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="J26" s="1" t="str">
+      <c r="J26" s="25" t="str">
         <f>F26</f>
         <v>MATH 325
 Intermediate Stats 
@@ -1979,28 +2224,43 @@
 Remote</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" s="8">
         <v>0.59375</v>
       </c>
+      <c r="B27" s="26"/>
       <c r="D27" s="1"/>
+      <c r="E27" s="26"/>
+      <c r="F27" s="26"/>
       <c r="H27" s="1"/>
-    </row>
-    <row r="28">
+      <c r="I27" s="26"/>
+      <c r="J27" s="26"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="8">
-        <v>0.6041666666666666</v>
-      </c>
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="B28" s="26"/>
       <c r="D28" s="1"/>
+      <c r="E28" s="26"/>
+      <c r="F28" s="26"/>
       <c r="H28" s="1"/>
-    </row>
-    <row r="29">
+      <c r="I28" s="26"/>
+      <c r="J28" s="26"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="8">
-        <v>0.6145833333333334</v>
-      </c>
+        <v>0.61458333333333337</v>
+      </c>
+      <c r="B29" s="26"/>
       <c r="D29" s="1"/>
+      <c r="E29" s="26"/>
+      <c r="F29" s="26"/>
       <c r="H29" s="1"/>
-    </row>
-    <row r="30">
+      <c r="I29" s="26"/>
+      <c r="J29" s="26"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="8">
         <v>0.625</v>
       </c>
@@ -2014,9 +2274,9 @@
       <c r="I30" s="4"/>
       <c r="J30" s="4"/>
     </row>
-    <row r="31">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" s="8">
-        <v>0.6354166666666666</v>
+        <v>0.63541666666666663</v>
       </c>
       <c r="B31" s="5"/>
       <c r="C31" s="5"/>
@@ -2028,9 +2288,9 @@
       <c r="I31" s="5"/>
       <c r="J31" s="5"/>
     </row>
-    <row r="32">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" s="8">
-        <v>0.6458333333333334</v>
+        <v>0.64583333333333337</v>
       </c>
       <c r="B32" s="5"/>
       <c r="C32" s="5"/>
@@ -2042,7 +2302,7 @@
       <c r="I32" s="5"/>
       <c r="J32" s="5"/>
     </row>
-    <row r="33">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" s="8">
         <v>0.65625</v>
       </c>
@@ -2056,9 +2316,9 @@
       <c r="I33" s="5"/>
       <c r="J33" s="5"/>
     </row>
-    <row r="34">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" s="8">
-        <v>0.6666666666666666</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="B34" s="5"/>
       <c r="C34" s="5"/>
@@ -2070,9 +2330,9 @@
       <c r="I34" s="5"/>
       <c r="J34" s="5"/>
     </row>
-    <row r="35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" s="8">
-        <v>0.6770833333333334</v>
+        <v>0.67708333333333337</v>
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="4"/>
@@ -2086,12 +2346,12 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="H2:H7"/>
-    <mergeCell ref="H9:H14"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="F16:F19"/>
+    <mergeCell ref="J16:J19"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="F26:F29"/>
+    <mergeCell ref="J26:J29"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="D2:D7"/>
     <mergeCell ref="D9:D14"/>
@@ -2099,476 +2359,478 @@
     <mergeCell ref="E26:E29"/>
     <mergeCell ref="I21:I24"/>
     <mergeCell ref="I26:I29"/>
+    <mergeCell ref="G11:G14"/>
+    <mergeCell ref="H2:H7"/>
+    <mergeCell ref="H9:H14"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:I1"/>
     <mergeCell ref="C11:C14"/>
-    <mergeCell ref="G11:G14"/>
-    <mergeCell ref="B16:B19"/>
-    <mergeCell ref="F16:F19"/>
-    <mergeCell ref="J16:J19"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="F26:F29"/>
-    <mergeCell ref="J26:J29"/>
   </mergeCells>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
+  <dimension ref="A1:F31"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="31.14"/>
-    <col customWidth="1" min="3" max="3" width="2.29"/>
-    <col customWidth="1" min="4" max="4" width="25.14"/>
-    <col customWidth="1" min="5" max="5" width="51.71"/>
+    <col min="2" max="2" width="31.140625" customWidth="1"/>
+    <col min="3" max="3" width="2.28515625" customWidth="1"/>
+    <col min="4" max="4" width="25.140625" customWidth="1"/>
+    <col min="5" max="5" width="51.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="C1" s="17">
-        <v>1.0</v>
-      </c>
-      <c r="D1" s="17" t="s">
+      <c r="C1" s="15">
+        <v>1</v>
+      </c>
+      <c r="D1" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="15" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="16" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="C2" s="19">
-        <v>1.0</v>
-      </c>
-      <c r="D2" s="19" t="s">
+      <c r="C2" s="17">
+        <v>1</v>
+      </c>
+      <c r="D2" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="E2" s="20" t="s">
+      <c r="E2" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="F2" s="19" t="s">
+      <c r="F2" s="17" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="16" t="s">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="C3" s="17">
-        <v>1.0</v>
-      </c>
-      <c r="D3" s="17" t="s">
+      <c r="C3" s="15">
+        <v>1</v>
+      </c>
+      <c r="D3" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="F3" s="17" t="s">
+      <c r="F3" s="15" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="16" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="B4" s="17" t="s">
         <v>57</v>
       </c>
-      <c r="C4" s="19">
-        <v>1.0</v>
-      </c>
-      <c r="D4" s="19" t="s">
+      <c r="C4" s="17">
+        <v>1</v>
+      </c>
+      <c r="D4" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="E4" s="20" t="s">
+      <c r="E4" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="17" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="21" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="C5" s="19">
-        <v>1.0</v>
-      </c>
-      <c r="D5" s="19" t="s">
+      <c r="C5" s="17">
+        <v>1</v>
+      </c>
+      <c r="D5" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="F5" s="18" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="21" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A6" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="B6" s="19" t="s">
+      <c r="B6" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="C6" s="19">
-        <v>1.0</v>
-      </c>
-      <c r="D6" s="19" t="s">
+      <c r="C6" s="17">
+        <v>1</v>
+      </c>
+      <c r="D6" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="E6" s="20" t="s">
+      <c r="E6" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="F6" s="20" t="s">
+      <c r="F6" s="18" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="22" t="s">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="C10" s="23">
-        <v>2.0</v>
-      </c>
-      <c r="D10" s="23" t="s">
+      <c r="C10" s="21">
+        <v>2</v>
+      </c>
+      <c r="D10" s="21" t="s">
         <v>72</v>
       </c>
-      <c r="E10" s="24" t="s">
+      <c r="E10" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="F10" s="23" t="s">
+      <c r="F10" s="21" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="22" t="s">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A11" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="B11" s="25" t="s">
+      <c r="B11" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="C11" s="25">
-        <v>2.0</v>
-      </c>
-      <c r="D11" s="25" t="s">
+      <c r="C11" s="23">
+        <v>2</v>
+      </c>
+      <c r="D11" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="E11" s="26" t="s">
+      <c r="E11" s="24" t="s">
         <v>76</v>
       </c>
-      <c r="F11" s="25" t="s">
+      <c r="F11" s="23" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="22" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A12" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="B12" s="23" t="s">
+      <c r="B12" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="C12" s="23">
-        <v>2.0</v>
-      </c>
-      <c r="D12" s="23" t="s">
+      <c r="C12" s="21">
+        <v>2</v>
+      </c>
+      <c r="D12" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="E12" s="24" t="s">
+      <c r="E12" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="F12" s="24" t="s">
+      <c r="F12" s="22" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="22" t="s">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="C13" s="25">
-        <v>2.0</v>
-      </c>
-      <c r="D13" s="25" t="s">
+      <c r="C13" s="23">
+        <v>2</v>
+      </c>
+      <c r="D13" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="E13" s="26" t="s">
+      <c r="E13" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="F13" s="25" t="s">
+      <c r="F13" s="23" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="22" t="s">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A14" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="B14" s="23" t="s">
+      <c r="B14" s="21" t="s">
         <v>71</v>
       </c>
-      <c r="C14" s="23">
-        <v>2.0</v>
-      </c>
-      <c r="D14" s="23" t="s">
+      <c r="C14" s="21">
+        <v>2</v>
+      </c>
+      <c r="D14" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="E14" s="24" t="s">
+      <c r="E14" s="22" t="s">
         <v>85</v>
       </c>
-      <c r="F14" s="23" t="s">
+      <c r="F14" s="21" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="22" t="s">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A15" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="B15" s="23" t="s">
+      <c r="B15" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="C15" s="23">
-        <v>3.0</v>
-      </c>
-      <c r="D15" s="23" t="s">
+      <c r="C15" s="21">
+        <v>3</v>
+      </c>
+      <c r="D15" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="E15" s="24" t="s">
+      <c r="E15" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="F15" s="24" t="s">
+      <c r="F15" s="22" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="22" t="s">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="23" t="s">
         <v>87</v>
       </c>
-      <c r="C16" s="25">
-        <v>3.0</v>
-      </c>
-      <c r="D16" s="25" t="s">
+      <c r="C16" s="23">
+        <v>3</v>
+      </c>
+      <c r="D16" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="E16" s="26" t="s">
+      <c r="E16" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="F16" s="24" t="s">
+      <c r="F16" s="22" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="22" t="s">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="B17" s="25" t="s">
+      <c r="B17" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="C17" s="25">
-        <v>1.0</v>
-      </c>
-      <c r="D17" s="25" t="s">
+      <c r="C17" s="23">
+        <v>1</v>
+      </c>
+      <c r="D17" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="E17" s="26" t="s">
+      <c r="E17" s="24" t="s">
         <v>94</v>
       </c>
-      <c r="F17" s="25" t="s">
+      <c r="F17" s="23" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="22" t="s">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="B18" s="23" t="s">
+      <c r="B18" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="C18" s="23">
-        <v>1.0</v>
-      </c>
-      <c r="D18" s="23" t="s">
+      <c r="C18" s="21">
+        <v>1</v>
+      </c>
+      <c r="D18" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="E18" s="24" t="s">
+      <c r="E18" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="F18" s="23" t="s">
+      <c r="F18" s="21" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="22" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="B19" s="25" t="s">
+      <c r="B19" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="C19" s="25">
-        <v>3.0</v>
-      </c>
-      <c r="D19" s="25" t="s">
+      <c r="C19" s="23">
+        <v>3</v>
+      </c>
+      <c r="D19" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="E19" s="26" t="s">
+      <c r="E19" s="24" t="s">
         <v>100</v>
       </c>
-      <c r="F19" s="24" t="s">
+      <c r="F19" s="22" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="22" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A20" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="C20" s="23">
-        <v>3.0</v>
-      </c>
-      <c r="D20" s="23" t="s">
+      <c r="C20" s="21">
+        <v>3</v>
+      </c>
+      <c r="D20" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="E20" s="24" t="s">
+      <c r="E20" s="22" t="s">
         <v>91</v>
       </c>
-      <c r="F20" s="24" t="s">
+      <c r="F20" s="22" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="22" t="s">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="B21" s="23" t="s">
+      <c r="B21" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="C21" s="23">
-        <v>3.0</v>
-      </c>
-      <c r="D21" s="23" t="s">
+      <c r="C21" s="21">
+        <v>3</v>
+      </c>
+      <c r="D21" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="E21" s="24" t="s">
+      <c r="E21" s="22" t="s">
         <v>105</v>
       </c>
-      <c r="F21" s="24" t="s">
+      <c r="F21" s="22" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="22"/>
-      <c r="B22" s="25"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="22" t="s">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" s="20"/>
+      <c r="B22" s="23"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="23"/>
+    </row>
+    <row r="29" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="B38" s="25" t="s">
+      <c r="B29" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="C38" s="25">
-        <v>3.0</v>
-      </c>
-      <c r="D38" s="25" t="s">
+      <c r="C29" s="23">
+        <v>3</v>
+      </c>
+      <c r="D29" s="23" t="s">
         <v>108</v>
       </c>
-      <c r="E38" s="26" t="s">
+      <c r="E29" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="F38" s="25" t="s">
+      <c r="F29" s="23" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="22" t="s">
+    <row r="30" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="B39" s="23" t="s">
+      <c r="B30" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="C39" s="23">
-        <v>3.0</v>
-      </c>
-      <c r="D39" s="23" t="s">
+      <c r="C30" s="21">
+        <v>3</v>
+      </c>
+      <c r="D30" s="21" t="s">
         <v>111</v>
       </c>
-      <c r="E39" s="24" t="s">
+      <c r="E30" s="22" t="s">
         <v>112</v>
       </c>
-      <c r="F39" s="23" t="s">
+      <c r="F30" s="21" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="22" t="s">
+    <row r="31" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="20" t="s">
         <v>113</v>
       </c>
-      <c r="B40" s="25" t="s">
+      <c r="B31" s="23" t="s">
         <v>107</v>
       </c>
-      <c r="C40" s="25">
-        <v>3.0</v>
-      </c>
-      <c r="D40" s="25" t="s">
+      <c r="C31" s="23">
+        <v>3</v>
+      </c>
+      <c r="D31" s="23" t="s">
         <v>108</v>
       </c>
-      <c r="E40" s="26" t="s">
+      <c r="E31" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="F40" s="25" t="s">
+      <c r="F31" s="23" t="s">
         <v>53</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
+  <dimension ref="A1:F31"/>
+  <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="11.71"/>
+    <col min="1" max="1" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2585,7 +2847,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="8">
         <v>0.375</v>
       </c>
@@ -2595,9 +2857,9 @@
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="8">
-        <v>0.3854166666666667</v>
+        <v>0.38541666666666669</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -2605,9 +2867,9 @@
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="8">
-        <v>0.3958333333333333</v>
+        <v>0.39583333333333331</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -2615,7 +2877,7 @@
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="8">
         <v>0.40625</v>
       </c>
@@ -2625,9 +2887,9 @@
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
-    <row r="6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="8">
-        <v>0.4166666666666667</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -2635,44 +2897,53 @@
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
-    <row r="7">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="8">
-        <v>0.4270833333333333</v>
-      </c>
-      <c r="B7" s="1" t="s">
+        <v>0.42708333333333331</v>
+      </c>
+      <c r="B7" s="25" t="s">
         <v>115</v>
       </c>
       <c r="C7" s="4"/>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="25" t="s">
         <v>115</v>
       </c>
       <c r="E7" s="4"/>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="25" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="8">
         <v>0.4375</v>
       </c>
+      <c r="B8" s="26"/>
       <c r="C8" s="4"/>
+      <c r="D8" s="26"/>
       <c r="E8" s="4"/>
-    </row>
-    <row r="9">
+      <c r="F8" s="26"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="8">
-        <v>0.4479166666666667</v>
-      </c>
+        <v>0.44791666666666669</v>
+      </c>
+      <c r="B9" s="26"/>
       <c r="C9" s="4"/>
+      <c r="D9" s="26"/>
       <c r="E9" s="4"/>
-    </row>
-    <row r="10">
+      <c r="F9" s="26"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="8">
-        <v>0.4583333333333333</v>
-      </c>
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="B10" s="26"/>
       <c r="C10" s="4"/>
+      <c r="D10" s="26"/>
       <c r="E10" s="4"/>
-    </row>
-    <row r="11">
+      <c r="F10" s="26"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="8">
         <v>0.46875</v>
       </c>
@@ -2682,49 +2953,49 @@
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
     </row>
-    <row r="12">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="8">
-        <v>0.4791666666666667</v>
-      </c>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-    </row>
-    <row r="13">
+        <v>0.47916666666666669</v>
+      </c>
+      <c r="B12" s="12"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="8">
-        <v>0.4895833333333333</v>
-      </c>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="13"/>
-    </row>
-    <row r="14">
+        <v>0.48958333333333331</v>
+      </c>
+      <c r="B13" s="12"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="8">
         <v>0.5</v>
       </c>
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-    </row>
-    <row r="15">
+      <c r="B14" s="12"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="8">
-        <v>0.5104166666666666</v>
-      </c>
-      <c r="B15" s="13"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
-    </row>
-    <row r="16">
+        <v>0.51041666666666663</v>
+      </c>
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="8">
-        <v>0.5208333333333334</v>
+        <v>0.52083333333333337</v>
       </c>
       <c r="B16" s="4"/>
       <c r="C16" s="4"/>
@@ -2732,7 +3003,7 @@
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
     </row>
-    <row r="17">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="8">
         <v>0.53125</v>
       </c>
@@ -2742,9 +3013,9 @@
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
     </row>
-    <row r="18">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="8">
-        <v>0.5416666666666666</v>
+        <v>0.54166666666666663</v>
       </c>
       <c r="B18" s="4"/>
       <c r="C18" s="4"/>
@@ -2752,9 +3023,9 @@
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
     </row>
-    <row r="19">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="8">
-        <v>0.5520833333333334</v>
+        <v>0.55208333333333337</v>
       </c>
       <c r="B19" s="4"/>
       <c r="C19" s="4"/>
@@ -2762,7 +3033,7 @@
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
     </row>
-    <row r="20">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="8">
         <v>0.5625</v>
       </c>
@@ -2772,9 +3043,9 @@
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
     </row>
-    <row r="21">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="8">
-        <v>0.5729166666666666</v>
+        <v>0.57291666666666663</v>
       </c>
       <c r="B21" s="4"/>
       <c r="C21" s="4"/>
@@ -2782,44 +3053,53 @@
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
     </row>
-    <row r="22">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="8">
-        <v>0.5833333333333334</v>
-      </c>
-      <c r="B22" s="1" t="s">
+        <v>0.58333333333333337</v>
+      </c>
+      <c r="B22" s="25" t="s">
         <v>116</v>
       </c>
       <c r="C22" s="4"/>
-      <c r="D22" s="1" t="s">
+      <c r="D22" s="25" t="s">
         <v>116</v>
       </c>
       <c r="E22" s="4"/>
-      <c r="F22" s="1" t="s">
+      <c r="F22" s="25" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="8">
         <v>0.59375</v>
       </c>
+      <c r="B23" s="26"/>
       <c r="C23" s="4"/>
+      <c r="D23" s="26"/>
       <c r="E23" s="4"/>
-    </row>
-    <row r="24">
+      <c r="F23" s="26"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="8">
-        <v>0.6041666666666666</v>
-      </c>
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="B24" s="26"/>
       <c r="C24" s="4"/>
+      <c r="D24" s="26"/>
       <c r="E24" s="4"/>
-    </row>
-    <row r="25">
+      <c r="F24" s="26"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="8">
-        <v>0.6145833333333334</v>
-      </c>
+        <v>0.61458333333333337</v>
+      </c>
+      <c r="B25" s="26"/>
       <c r="C25" s="4"/>
+      <c r="D25" s="26"/>
       <c r="E25" s="4"/>
-    </row>
-    <row r="26">
+      <c r="F25" s="26"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="8">
         <v>0.625</v>
       </c>
@@ -2831,46 +3111,55 @@
       <c r="E26" s="4"/>
       <c r="F26" s="4"/>
     </row>
-    <row r="27">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="8">
-        <v>0.6354166666666666</v>
-      </c>
-      <c r="B27" s="5" t="s">
+        <v>0.63541666666666663</v>
+      </c>
+      <c r="B27" s="27" t="s">
         <v>117</v>
       </c>
       <c r="C27" s="6"/>
-      <c r="D27" s="5" t="s">
+      <c r="D27" s="27" t="s">
         <v>117</v>
       </c>
       <c r="E27" s="6"/>
-      <c r="F27" s="5" t="s">
+      <c r="F27" s="27" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="8">
-        <v>0.6458333333333334</v>
-      </c>
+        <v>0.64583333333333337</v>
+      </c>
+      <c r="B28" s="26"/>
       <c r="C28" s="6"/>
+      <c r="D28" s="26"/>
       <c r="E28" s="6"/>
-    </row>
-    <row r="29">
+      <c r="F28" s="26"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="8">
         <v>0.65625</v>
       </c>
+      <c r="B29" s="26"/>
       <c r="C29" s="6"/>
+      <c r="D29" s="26"/>
       <c r="E29" s="6"/>
-    </row>
-    <row r="30">
+      <c r="F29" s="26"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="8">
-        <v>0.6666666666666666</v>
-      </c>
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="B30" s="26"/>
       <c r="C30" s="6"/>
+      <c r="D30" s="26"/>
       <c r="E30" s="6"/>
-    </row>
-    <row r="31">
+      <c r="F30" s="26"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="8">
-        <v>0.6770833333333334</v>
+        <v>0.67708333333333337</v>
       </c>
       <c r="B31" s="4"/>
       <c r="C31" s="4"/>
@@ -2890,6 +3179,6 @@
     <mergeCell ref="B27:B30"/>
     <mergeCell ref="D27:D30"/>
   </mergeCells>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update at 17:15 on 07/27/2020
</commit_message>
<xml_diff>
--- a/site_libs/fall 2020.xlsx
+++ b/site_libs/fall 2020.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Portfolio\site_libs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB4EB6CB-43A5-4CC7-8A1A-80231397519D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19DB343C-07C6-4022-B398-3CAE05446461}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Schedule" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="124">
   <si>
     <t>Monday</t>
   </si>
@@ -429,13 +429,18 @@
   </si>
   <si>
     <t>CSE 121b JavaScript Barney Remote</t>
+  </si>
+  <si>
+    <t>TA 
+ECEN 361
+Grimmett</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -497,6 +502,20 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF0076B6"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF020202"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -530,7 +549,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -590,30 +609,36 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -856,26 +881,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="B1" s="25" t="s">
+      <c r="B1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="26"/>
-      <c r="D1" s="25" t="s">
+      <c r="C1" s="31"/>
+      <c r="D1" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="26"/>
-      <c r="F1" s="25" t="s">
+      <c r="E1" s="31"/>
+      <c r="F1" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="26"/>
-      <c r="H1" s="25" t="s">
+      <c r="G1" s="31"/>
+      <c r="H1" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="26"/>
-      <c r="J1" s="25" t="s">
+      <c r="I1" s="31"/>
+      <c r="J1" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="26"/>
+      <c r="K1" s="31"/>
       <c r="L1" s="1"/>
       <c r="M1" s="2" t="s">
         <v>5</v>
@@ -910,7 +935,7 @@
         <v>0.32291666666666669</v>
       </c>
       <c r="B2" s="4"/>
-      <c r="C2" s="31"/>
+      <c r="C2" s="25"/>
       <c r="D2" s="6"/>
       <c r="E2" s="6"/>
       <c r="F2" s="6"/>
@@ -953,14 +978,14 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="B3" s="4"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="27" t="s">
+      <c r="C3" s="25"/>
+      <c r="D3" s="30" t="s">
         <v>20</v>
       </c>
       <c r="E3" s="6"/>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
-      <c r="H3" s="27" t="str">
+      <c r="H3" s="30" t="str">
         <f>D3</f>
         <v>MATH 488
 Consulting
@@ -1004,12 +1029,12 @@
         <v>0.34375</v>
       </c>
       <c r="B4" s="4"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="32"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="27"/>
       <c r="E4" s="6"/>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
-      <c r="H4" s="32"/>
+      <c r="H4" s="27"/>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -1047,12 +1072,12 @@
         <v>0.35416666666666669</v>
       </c>
       <c r="B5" s="4"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="32"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="27"/>
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
-      <c r="H5" s="32"/>
+      <c r="H5" s="27"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -1090,12 +1115,12 @@
         <v>0.36458333333333331</v>
       </c>
       <c r="B6" s="4"/>
-      <c r="C6" s="31"/>
-      <c r="D6" s="32"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="27"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
-      <c r="H6" s="32"/>
+      <c r="H6" s="27"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -1110,12 +1135,12 @@
         <v>0.375</v>
       </c>
       <c r="B7" s="4"/>
-      <c r="C7" s="31"/>
-      <c r="D7" s="32"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="27"/>
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
-      <c r="H7" s="32"/>
+      <c r="H7" s="27"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -1126,12 +1151,12 @@
         <v>0.38541666666666669</v>
       </c>
       <c r="B8" s="4"/>
-      <c r="C8" s="31"/>
-      <c r="D8" s="32"/>
+      <c r="C8" s="25"/>
+      <c r="D8" s="27"/>
       <c r="E8" s="6"/>
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
-      <c r="H8" s="32"/>
+      <c r="H8" s="27"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4"/>
       <c r="K8" s="4"/>
@@ -1142,7 +1167,7 @@
         <v>0.39583333333333331</v>
       </c>
       <c r="B9" s="4"/>
-      <c r="C9" s="31"/>
+      <c r="C9" s="25"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
@@ -1161,7 +1186,7 @@
         <v>0.40625</v>
       </c>
       <c r="B10" s="4"/>
-      <c r="C10" s="31"/>
+      <c r="C10" s="25"/>
       <c r="D10" s="11"/>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
@@ -1180,7 +1205,7 @@
         <v>0.41666666666666669</v>
       </c>
       <c r="B11" s="4"/>
-      <c r="C11" s="31"/>
+      <c r="C11" s="25"/>
       <c r="D11" s="11"/>
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
@@ -1199,7 +1224,7 @@
       <c r="C12" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="33" t="s">
+      <c r="D12" s="28" t="s">
         <v>122</v>
       </c>
       <c r="E12" s="4"/>
@@ -1207,64 +1232,64 @@
       <c r="G12" s="29" t="s">
         <v>35</v>
       </c>
-      <c r="H12" s="33" t="s">
+      <c r="H12" s="28" t="s">
         <v>122</v>
       </c>
       <c r="I12" s="4"/>
       <c r="J12" s="4"/>
-      <c r="K12" s="31"/>
+      <c r="K12" s="25"/>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A13" s="8">
         <v>0.4375</v>
       </c>
       <c r="B13" s="4"/>
-      <c r="C13" s="32"/>
-      <c r="D13" s="33"/>
+      <c r="C13" s="27"/>
+      <c r="D13" s="28"/>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
-      <c r="G13" s="32"/>
-      <c r="H13" s="33"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="28"/>
       <c r="I13" s="4"/>
       <c r="J13" s="4"/>
-      <c r="K13" s="31"/>
+      <c r="K13" s="25"/>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A14" s="8">
         <v>0.44791666666666669</v>
       </c>
       <c r="B14" s="4"/>
-      <c r="C14" s="32"/>
-      <c r="D14" s="33"/>
+      <c r="C14" s="27"/>
+      <c r="D14" s="28"/>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
-      <c r="G14" s="32"/>
-      <c r="H14" s="33"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="28"/>
       <c r="I14" s="4"/>
       <c r="J14" s="4"/>
-      <c r="K14" s="31"/>
+      <c r="K14" s="25"/>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A15" s="8">
         <v>0.45833333333333331</v>
       </c>
       <c r="B15" s="4"/>
-      <c r="C15" s="32"/>
-      <c r="D15" s="33"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="28"/>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
-      <c r="G15" s="32"/>
-      <c r="H15" s="33"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="28"/>
       <c r="I15" s="4"/>
       <c r="J15" s="4"/>
-      <c r="K15" s="31"/>
+      <c r="K15" s="25"/>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A16" s="8">
         <v>0.46875</v>
       </c>
       <c r="B16" s="4"/>
-      <c r="C16" s="31"/>
+      <c r="C16" s="25"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
@@ -1272,19 +1297,19 @@
       <c r="H16" s="4"/>
       <c r="I16" s="4"/>
       <c r="J16" s="4"/>
-      <c r="K16" s="31"/>
+      <c r="K16" s="25"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" s="8">
         <v>0.47916666666666669</v>
       </c>
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="C17" s="31"/>
+      <c r="C17" s="25"/>
       <c r="D17" s="12"/>
       <c r="E17" s="12"/>
-      <c r="F17" s="27" t="str">
+      <c r="F17" s="30" t="str">
         <f>B17</f>
         <v>CSE 450
 Machine Learning
@@ -1294,66 +1319,66 @@
       <c r="G17" s="12"/>
       <c r="H17" s="12"/>
       <c r="I17" s="12"/>
-      <c r="J17" s="27" t="str">
+      <c r="J17" s="30" t="str">
         <f>F17</f>
         <v>CSE 450
 Machine Learning
 Burton 
 STC  394</v>
       </c>
-      <c r="K17" s="31"/>
+      <c r="K17" s="25"/>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" s="8">
         <v>0.48958333333333331</v>
       </c>
-      <c r="B18" s="32"/>
-      <c r="C18" s="31"/>
+      <c r="B18" s="27"/>
+      <c r="C18" s="25"/>
       <c r="D18" s="12"/>
       <c r="E18" s="12"/>
-      <c r="F18" s="32"/>
+      <c r="F18" s="27"/>
       <c r="G18" s="12"/>
       <c r="H18" s="12"/>
       <c r="I18" s="12"/>
-      <c r="J18" s="32"/>
-      <c r="K18" s="31"/>
+      <c r="J18" s="27"/>
+      <c r="K18" s="25"/>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" s="8">
         <v>0.5</v>
       </c>
-      <c r="B19" s="32"/>
-      <c r="C19" s="31"/>
+      <c r="B19" s="27"/>
+      <c r="C19" s="25"/>
       <c r="D19" s="12"/>
       <c r="E19" s="12"/>
-      <c r="F19" s="32"/>
+      <c r="F19" s="27"/>
       <c r="G19" s="12"/>
       <c r="H19" s="12"/>
       <c r="I19" s="12"/>
-      <c r="J19" s="32"/>
-      <c r="K19" s="31"/>
+      <c r="J19" s="27"/>
+      <c r="K19" s="25"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" s="8">
         <v>0.51041666666666663</v>
       </c>
-      <c r="B20" s="32"/>
-      <c r="C20" s="31"/>
+      <c r="B20" s="27"/>
+      <c r="C20" s="25"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
-      <c r="F20" s="32"/>
+      <c r="F20" s="27"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
       <c r="I20" s="4"/>
-      <c r="J20" s="32"/>
-      <c r="K20" s="31"/>
+      <c r="J20" s="27"/>
+      <c r="K20" s="25"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" s="8">
         <v>0.52083333333333337</v>
       </c>
       <c r="B21" s="4"/>
-      <c r="C21" s="31"/>
+      <c r="C21" s="25"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
@@ -1361,181 +1386,181 @@
       <c r="H21" s="4"/>
       <c r="I21" s="4"/>
       <c r="J21" s="4"/>
-      <c r="K21" s="31"/>
+      <c r="K21" s="25"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" s="8">
         <v>0.53125</v>
       </c>
-      <c r="B22" s="4"/>
-      <c r="C22" s="31"/>
+      <c r="C22" s="29" t="s">
+        <v>123</v>
+      </c>
       <c r="D22" s="4"/>
       <c r="E22" s="29" t="s">
         <v>34</v>
       </c>
       <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
+      <c r="G22" s="29" t="s">
+        <v>123</v>
+      </c>
       <c r="H22" s="4"/>
       <c r="I22" s="29" t="s">
         <v>35</v>
       </c>
       <c r="J22" s="4"/>
-      <c r="K22" s="31"/>
+      <c r="K22" s="25"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" s="8">
         <v>0.54166666666666663</v>
       </c>
-      <c r="B23" s="4"/>
-      <c r="C23" s="31"/>
+      <c r="C23" s="27"/>
       <c r="D23" s="4"/>
-      <c r="E23" s="32"/>
+      <c r="E23" s="27"/>
       <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
+      <c r="G23" s="27"/>
       <c r="H23" s="4"/>
-      <c r="I23" s="32"/>
+      <c r="I23" s="27"/>
       <c r="J23" s="4"/>
-      <c r="K23" s="31"/>
+      <c r="K23" s="25"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" s="8">
         <v>0.55208333333333337</v>
       </c>
-      <c r="B24" s="4"/>
-      <c r="C24" s="31"/>
+      <c r="C24" s="27"/>
       <c r="D24" s="4"/>
-      <c r="E24" s="32"/>
+      <c r="E24" s="27"/>
       <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
+      <c r="G24" s="27"/>
       <c r="H24" s="4"/>
-      <c r="I24" s="32"/>
+      <c r="I24" s="27"/>
       <c r="J24" s="4"/>
-      <c r="K24" s="31"/>
+      <c r="K24" s="25"/>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" s="8">
         <v>0.5625</v>
       </c>
-      <c r="B25" s="4"/>
-      <c r="C25" s="31"/>
+      <c r="C25" s="27"/>
       <c r="D25" s="4"/>
-      <c r="E25" s="32"/>
+      <c r="E25" s="27"/>
       <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
+      <c r="G25" s="27"/>
       <c r="H25" s="4"/>
-      <c r="I25" s="32"/>
+      <c r="I25" s="27"/>
       <c r="J25" s="4"/>
-      <c r="K25" s="31"/>
+      <c r="K25" s="25"/>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" s="8">
         <v>0.57291666666666663</v>
       </c>
-      <c r="B26" s="31"/>
-      <c r="C26" s="31"/>
-      <c r="D26" s="31"/>
-      <c r="E26" s="31"/>
-      <c r="F26" s="31"/>
-      <c r="G26" s="31"/>
-      <c r="H26" s="31"/>
-      <c r="I26" s="31"/>
-      <c r="J26" s="31"/>
-      <c r="K26" s="31"/>
+      <c r="B26" s="25"/>
+      <c r="C26" s="25"/>
+      <c r="D26" s="25"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="25"/>
+      <c r="G26" s="25"/>
+      <c r="H26" s="25"/>
+      <c r="I26" s="25"/>
+      <c r="J26" s="25"/>
+      <c r="K26" s="25"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" s="8">
         <v>0.58333333333333337</v>
       </c>
-      <c r="B27" s="25" t="s">
+      <c r="B27" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="C27" s="31"/>
+      <c r="C27" s="25"/>
       <c r="D27" s="4"/>
       <c r="E27" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="F27" s="25" t="str">
+      <c r="F27" s="26" t="str">
         <f>B27</f>
         <v>MATH 325
 Intermediate Stats 
 Saunders 
 Remote</v>
       </c>
-      <c r="G27" s="31"/>
+      <c r="G27" s="25"/>
       <c r="H27" s="4"/>
       <c r="I27" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="J27" s="25" t="str">
+      <c r="J27" s="26" t="str">
         <f>F27</f>
         <v>MATH 325
 Intermediate Stats 
 Saunders 
 Remote</v>
       </c>
-      <c r="K27" s="31"/>
+      <c r="K27" s="25"/>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A28" s="8">
         <v>0.59375</v>
       </c>
-      <c r="B28" s="32"/>
-      <c r="C28" s="31"/>
+      <c r="B28" s="27"/>
+      <c r="C28" s="25"/>
       <c r="D28" s="4"/>
-      <c r="E28" s="32"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="31"/>
+      <c r="E28" s="27"/>
+      <c r="F28" s="27"/>
+      <c r="G28" s="25"/>
       <c r="H28" s="4"/>
-      <c r="I28" s="32"/>
-      <c r="J28" s="32"/>
-      <c r="K28" s="31"/>
+      <c r="I28" s="27"/>
+      <c r="J28" s="27"/>
+      <c r="K28" s="25"/>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" s="8">
         <v>0.60416666666666663</v>
       </c>
-      <c r="B29" s="32"/>
-      <c r="C29" s="31"/>
+      <c r="B29" s="27"/>
+      <c r="C29" s="25"/>
       <c r="D29" s="4"/>
-      <c r="E29" s="32"/>
-      <c r="F29" s="32"/>
-      <c r="G29" s="31"/>
+      <c r="E29" s="27"/>
+      <c r="F29" s="27"/>
+      <c r="G29" s="25"/>
       <c r="H29" s="4"/>
-      <c r="I29" s="32"/>
-      <c r="J29" s="32"/>
-      <c r="K29" s="31"/>
+      <c r="I29" s="27"/>
+      <c r="J29" s="27"/>
+      <c r="K29" s="25"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="8">
         <v>0.61458333333333337</v>
       </c>
-      <c r="B30" s="32"/>
-      <c r="C30" s="31"/>
+      <c r="B30" s="27"/>
+      <c r="C30" s="25"/>
       <c r="D30" s="4"/>
-      <c r="E30" s="32"/>
-      <c r="F30" s="32"/>
-      <c r="G30" s="31"/>
+      <c r="E30" s="27"/>
+      <c r="F30" s="27"/>
+      <c r="G30" s="25"/>
       <c r="H30" s="4"/>
-      <c r="I30" s="32"/>
-      <c r="J30" s="32"/>
-      <c r="K30" s="31"/>
+      <c r="I30" s="27"/>
+      <c r="J30" s="27"/>
+      <c r="K30" s="25"/>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" s="8">
         <v>0.625</v>
       </c>
       <c r="B31" s="4"/>
-      <c r="C31" s="31"/>
+      <c r="C31" s="25"/>
       <c r="D31" s="4"/>
       <c r="E31" s="4"/>
       <c r="F31" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="G31" s="31"/>
+      <c r="G31" s="25"/>
       <c r="H31" s="4"/>
       <c r="I31" s="4"/>
       <c r="J31" s="4"/>
-      <c r="K31" s="31"/>
+      <c r="K31" s="25"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" s="8">
@@ -1550,7 +1575,7 @@
       <c r="H32" s="6"/>
       <c r="I32" s="6"/>
       <c r="J32" s="6"/>
-      <c r="K32" s="31"/>
+      <c r="K32" s="25"/>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A33" s="8">
@@ -1565,7 +1590,7 @@
       <c r="H33" s="6"/>
       <c r="I33" s="6"/>
       <c r="J33" s="6"/>
-      <c r="K33" s="31"/>
+      <c r="K33" s="25"/>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" s="8">
@@ -1580,7 +1605,7 @@
       <c r="H34" s="6"/>
       <c r="I34" s="6"/>
       <c r="J34" s="6"/>
-      <c r="K34" s="31"/>
+      <c r="K34" s="25"/>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" s="8">
@@ -1595,7 +1620,7 @@
       <c r="H35" s="6"/>
       <c r="I35" s="6"/>
       <c r="J35" s="6"/>
-      <c r="K35" s="31"/>
+      <c r="K35" s="25"/>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A36" s="8">
@@ -1610,10 +1635,22 @@
       <c r="H36" s="4"/>
       <c r="I36" s="4"/>
       <c r="J36" s="4"/>
-      <c r="K36" s="31"/>
+      <c r="K36" s="25"/>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="23">
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="D3:D8"/>
+    <mergeCell ref="H3:H8"/>
+    <mergeCell ref="E22:E25"/>
+    <mergeCell ref="E27:E30"/>
+    <mergeCell ref="I22:I25"/>
+    <mergeCell ref="I27:I30"/>
+    <mergeCell ref="G22:G25"/>
     <mergeCell ref="B27:B30"/>
     <mergeCell ref="F27:F30"/>
     <mergeCell ref="J27:J30"/>
@@ -1624,17 +1661,7 @@
     <mergeCell ref="B17:B20"/>
     <mergeCell ref="F17:F20"/>
     <mergeCell ref="J17:J20"/>
-    <mergeCell ref="D3:D8"/>
-    <mergeCell ref="H3:H8"/>
-    <mergeCell ref="E22:E25"/>
-    <mergeCell ref="E27:E30"/>
-    <mergeCell ref="I22:I25"/>
-    <mergeCell ref="I27:I30"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="C22:C25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1668,26 +1695,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="B1" s="25" t="s">
+      <c r="B1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="26"/>
-      <c r="D1" s="25" t="s">
+      <c r="C1" s="31"/>
+      <c r="D1" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="26"/>
-      <c r="F1" s="25" t="s">
+      <c r="E1" s="31"/>
+      <c r="F1" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="26"/>
-      <c r="H1" s="25" t="s">
+      <c r="G1" s="31"/>
+      <c r="H1" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="I1" s="26"/>
-      <c r="J1" s="25" t="s">
+      <c r="I1" s="31"/>
+      <c r="J1" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="26"/>
+      <c r="K1" s="31"/>
       <c r="L1" s="1"/>
       <c r="M1" s="2" t="s">
         <v>5</v>
@@ -1722,13 +1749,13 @@
         <v>0.33333333333333331</v>
       </c>
       <c r="B2" s="4"/>
-      <c r="D2" s="30" t="s">
+      <c r="D2" s="32" t="s">
         <v>40</v>
       </c>
       <c r="E2" s="4"/>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
-      <c r="H2" s="30" t="str">
+      <c r="H2" s="32" t="str">
         <f>D2</f>
         <v>CSE 341
 Web Backend 2
@@ -1772,11 +1799,11 @@
         <v>0.34375</v>
       </c>
       <c r="B3" s="4"/>
-      <c r="D3" s="26"/>
+      <c r="D3" s="31"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
-      <c r="H3" s="26"/>
+      <c r="H3" s="31"/>
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
@@ -1814,11 +1841,11 @@
         <v>0.35416666666666669</v>
       </c>
       <c r="B4" s="4"/>
-      <c r="D4" s="26"/>
+      <c r="D4" s="31"/>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
-      <c r="H4" s="26"/>
+      <c r="H4" s="31"/>
       <c r="I4" s="4"/>
       <c r="J4" s="4"/>
       <c r="K4" s="4"/>
@@ -1856,11 +1883,11 @@
         <v>0.36458333333333331</v>
       </c>
       <c r="B5" s="4"/>
-      <c r="D5" s="26"/>
+      <c r="D5" s="31"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
-      <c r="H5" s="26"/>
+      <c r="H5" s="31"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
@@ -1898,11 +1925,11 @@
         <v>0.375</v>
       </c>
       <c r="B6" s="4"/>
-      <c r="D6" s="26"/>
+      <c r="D6" s="31"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
-      <c r="H6" s="26"/>
+      <c r="H6" s="31"/>
       <c r="I6" s="4"/>
       <c r="J6" s="4"/>
       <c r="K6" s="4"/>
@@ -1913,11 +1940,11 @@
         <v>0.38541666666666669</v>
       </c>
       <c r="B7" s="4"/>
-      <c r="D7" s="26"/>
+      <c r="D7" s="31"/>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
-      <c r="H7" s="26"/>
+      <c r="H7" s="31"/>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7" s="4"/>
@@ -1949,13 +1976,13 @@
         <v>0.40625</v>
       </c>
       <c r="B9" s="4"/>
-      <c r="D9" s="30" t="s">
+      <c r="D9" s="32" t="s">
         <v>48</v>
       </c>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
-      <c r="H9" s="30" t="s">
+      <c r="H9" s="32" t="s">
         <v>48</v>
       </c>
       <c r="I9" s="4"/>
@@ -1968,11 +1995,11 @@
         <v>0.41666666666666669</v>
       </c>
       <c r="B10" s="4"/>
-      <c r="D10" s="26"/>
+      <c r="D10" s="31"/>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
       <c r="G10" s="4"/>
-      <c r="H10" s="26"/>
+      <c r="H10" s="31"/>
       <c r="I10" s="4"/>
       <c r="J10" s="4"/>
       <c r="K10" s="4"/>
@@ -1983,19 +2010,19 @@
         <v>0.42708333333333331</v>
       </c>
       <c r="B11" s="1"/>
-      <c r="C11" s="28" t="s">
+      <c r="C11" s="33" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="26"/>
+      <c r="D11" s="31"/>
       <c r="E11" s="4"/>
       <c r="F11" s="1">
         <f>B11</f>
         <v>0</v>
       </c>
-      <c r="G11" s="28" t="s">
+      <c r="G11" s="33" t="s">
         <v>35</v>
       </c>
-      <c r="H11" s="26"/>
+      <c r="H11" s="31"/>
       <c r="I11" s="4"/>
       <c r="J11" s="1"/>
     </row>
@@ -2004,12 +2031,12 @@
         <v>0.4375</v>
       </c>
       <c r="B12" s="1"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
       <c r="E12" s="4"/>
       <c r="F12" s="1"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="26"/>
+      <c r="G12" s="31"/>
+      <c r="H12" s="31"/>
       <c r="I12" s="4"/>
       <c r="J12" s="1"/>
     </row>
@@ -2018,12 +2045,12 @@
         <v>0.44791666666666669</v>
       </c>
       <c r="B13" s="1"/>
-      <c r="C13" s="26"/>
-      <c r="D13" s="26"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
       <c r="E13" s="4"/>
       <c r="F13" s="1"/>
-      <c r="G13" s="26"/>
-      <c r="H13" s="26"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="31"/>
       <c r="I13" s="4"/>
       <c r="J13" s="1"/>
     </row>
@@ -2032,12 +2059,12 @@
         <v>0.45833333333333331</v>
       </c>
       <c r="B14" s="1"/>
-      <c r="C14" s="26"/>
-      <c r="D14" s="26"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="31"/>
       <c r="E14" s="4"/>
       <c r="F14" s="1"/>
-      <c r="G14" s="26"/>
-      <c r="H14" s="26"/>
+      <c r="G14" s="31"/>
+      <c r="H14" s="31"/>
       <c r="I14" s="4"/>
       <c r="J14" s="1"/>
     </row>
@@ -2058,12 +2085,12 @@
       <c r="A16" s="8">
         <v>0.47916666666666669</v>
       </c>
-      <c r="B16" s="27" t="s">
+      <c r="B16" s="30" t="s">
         <v>36</v>
       </c>
       <c r="D16" s="12"/>
       <c r="E16" s="12"/>
-      <c r="F16" s="27" t="str">
+      <c r="F16" s="30" t="str">
         <f>B16</f>
         <v>CSE 450
 Machine Learning
@@ -2073,7 +2100,7 @@
       <c r="G16" s="12"/>
       <c r="H16" s="12"/>
       <c r="I16" s="12"/>
-      <c r="J16" s="27" t="str">
+      <c r="J16" s="30" t="str">
         <f>F16</f>
         <v>CSE 450
 Machine Learning
@@ -2085,40 +2112,40 @@
       <c r="A17" s="8">
         <v>0.48958333333333331</v>
       </c>
-      <c r="B17" s="26"/>
+      <c r="B17" s="31"/>
       <c r="D17" s="12"/>
       <c r="E17" s="12"/>
-      <c r="F17" s="26"/>
+      <c r="F17" s="31"/>
       <c r="G17" s="12"/>
       <c r="H17" s="12"/>
       <c r="I17" s="12"/>
-      <c r="J17" s="26"/>
+      <c r="J17" s="31"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="8">
         <v>0.5</v>
       </c>
-      <c r="B18" s="26"/>
+      <c r="B18" s="31"/>
       <c r="D18" s="12"/>
       <c r="E18" s="12"/>
-      <c r="F18" s="26"/>
+      <c r="F18" s="31"/>
       <c r="G18" s="12"/>
       <c r="H18" s="12"/>
       <c r="I18" s="12"/>
-      <c r="J18" s="26"/>
+      <c r="J18" s="31"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="8">
         <v>0.51041666666666663</v>
       </c>
-      <c r="B19" s="26"/>
+      <c r="B19" s="31"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
-      <c r="F19" s="26"/>
+      <c r="F19" s="31"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
       <c r="I19" s="4"/>
-      <c r="J19" s="26"/>
+      <c r="J19" s="31"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="8">
@@ -2139,13 +2166,13 @@
       </c>
       <c r="B21" s="4"/>
       <c r="D21" s="4"/>
-      <c r="E21" s="28" t="s">
+      <c r="E21" s="33" t="s">
         <v>34</v>
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
-      <c r="I21" s="28" t="s">
+      <c r="I21" s="33" t="s">
         <v>35</v>
       </c>
       <c r="J21" s="4"/>
@@ -2156,11 +2183,11 @@
       </c>
       <c r="B22" s="4"/>
       <c r="D22" s="4"/>
-      <c r="E22" s="26"/>
+      <c r="E22" s="31"/>
       <c r="F22" s="4"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
-      <c r="I22" s="26"/>
+      <c r="I22" s="31"/>
       <c r="J22" s="4"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
@@ -2169,11 +2196,11 @@
       </c>
       <c r="B23" s="4"/>
       <c r="D23" s="4"/>
-      <c r="E23" s="26"/>
+      <c r="E23" s="31"/>
       <c r="F23" s="4"/>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
-      <c r="I23" s="26"/>
+      <c r="I23" s="31"/>
       <c r="J23" s="4"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
@@ -2182,11 +2209,11 @@
       </c>
       <c r="B24" s="4"/>
       <c r="D24" s="4"/>
-      <c r="E24" s="26"/>
+      <c r="E24" s="31"/>
       <c r="F24" s="4"/>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
-      <c r="I24" s="26"/>
+      <c r="I24" s="31"/>
       <c r="J24" s="4"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
@@ -2198,14 +2225,14 @@
       <c r="A26" s="8">
         <v>0.58333333333333337</v>
       </c>
-      <c r="B26" s="25" t="s">
+      <c r="B26" s="26" t="s">
         <v>37</v>
       </c>
       <c r="D26" s="1"/>
       <c r="E26" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="F26" s="25" t="str">
+      <c r="F26" s="26" t="str">
         <f>B26</f>
         <v>MATH 325
 Intermediate Stats 
@@ -2216,7 +2243,7 @@
       <c r="I26" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="J26" s="25" t="str">
+      <c r="J26" s="26" t="str">
         <f>F26</f>
         <v>MATH 325
 Intermediate Stats 
@@ -2228,37 +2255,37 @@
       <c r="A27" s="8">
         <v>0.59375</v>
       </c>
-      <c r="B27" s="26"/>
+      <c r="B27" s="31"/>
       <c r="D27" s="1"/>
-      <c r="E27" s="26"/>
-      <c r="F27" s="26"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="31"/>
       <c r="H27" s="1"/>
-      <c r="I27" s="26"/>
-      <c r="J27" s="26"/>
+      <c r="I27" s="31"/>
+      <c r="J27" s="31"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="8">
         <v>0.60416666666666663</v>
       </c>
-      <c r="B28" s="26"/>
+      <c r="B28" s="31"/>
       <c r="D28" s="1"/>
-      <c r="E28" s="26"/>
-      <c r="F28" s="26"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="31"/>
       <c r="H28" s="1"/>
-      <c r="I28" s="26"/>
-      <c r="J28" s="26"/>
+      <c r="I28" s="31"/>
+      <c r="J28" s="31"/>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="8">
         <v>0.61458333333333337</v>
       </c>
-      <c r="B29" s="26"/>
+      <c r="B29" s="31"/>
       <c r="D29" s="1"/>
-      <c r="E29" s="26"/>
-      <c r="F29" s="26"/>
+      <c r="E29" s="31"/>
+      <c r="F29" s="31"/>
       <c r="H29" s="1"/>
-      <c r="I29" s="26"/>
-      <c r="J29" s="26"/>
+      <c r="I29" s="31"/>
+      <c r="J29" s="31"/>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="8">
@@ -2346,12 +2373,11 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="B16:B19"/>
-    <mergeCell ref="F16:F19"/>
-    <mergeCell ref="J16:J19"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="F26:F29"/>
-    <mergeCell ref="J26:J29"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="C11:C14"/>
     <mergeCell ref="J1:K1"/>
     <mergeCell ref="D2:D7"/>
     <mergeCell ref="D9:D14"/>
@@ -2362,11 +2388,12 @@
     <mergeCell ref="G11:G14"/>
     <mergeCell ref="H2:H7"/>
     <mergeCell ref="H9:H14"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="H1:I1"/>
-    <mergeCell ref="C11:C14"/>
+    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="F16:F19"/>
+    <mergeCell ref="J16:J19"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="F26:F29"/>
+    <mergeCell ref="J26:J29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2380,13 +2407,13 @@
   <dimension ref="A1:F31"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="31.140625" customWidth="1"/>
+    <col min="2" max="2" width="32.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="2.28515625" customWidth="1"/>
     <col min="4" max="4" width="25.140625" customWidth="1"/>
     <col min="5" max="5" width="51.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A1" s="14" t="s">
         <v>49</v>
       </c>
@@ -2406,7 +2433,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A2" s="14" t="s">
         <v>54</v>
       </c>
@@ -2426,7 +2453,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A3" s="14" t="s">
         <v>56</v>
       </c>
@@ -2446,7 +2473,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A4" s="14" t="s">
         <v>59</v>
       </c>
@@ -2466,7 +2493,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A5" s="19" t="s">
         <v>61</v>
       </c>
@@ -2486,7 +2513,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A6" s="19" t="s">
         <v>66</v>
       </c>
@@ -2506,7 +2533,27 @@
         <v>69</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="35" t="s">
+        <v>104</v>
+      </c>
+      <c r="C7" s="35">
+        <v>3</v>
+      </c>
+      <c r="D7" s="35" t="s">
+        <v>51</v>
+      </c>
+      <c r="E7" s="35" t="s">
+        <v>105</v>
+      </c>
+      <c r="F7" s="35" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A10" s="20" t="s">
         <v>70</v>
       </c>
@@ -2526,7 +2573,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A11" s="20" t="s">
         <v>74</v>
       </c>
@@ -2546,7 +2593,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A12" s="20" t="s">
         <v>77</v>
       </c>
@@ -2566,7 +2613,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A13" s="20" t="s">
         <v>80</v>
       </c>
@@ -2586,7 +2633,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A14" s="20" t="s">
         <v>83</v>
       </c>
@@ -2606,7 +2653,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A15" s="20" t="s">
         <v>86</v>
       </c>
@@ -2626,7 +2673,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A16" s="20" t="s">
         <v>90</v>
       </c>
@@ -2646,7 +2693,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A17" s="20" t="s">
         <v>92</v>
       </c>
@@ -2666,7 +2713,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A18" s="20" t="s">
         <v>96</v>
       </c>
@@ -2686,7 +2733,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A19" s="20" t="s">
         <v>98</v>
       </c>
@@ -2706,7 +2753,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A20" s="20" t="s">
         <v>102</v>
       </c>
@@ -2726,27 +2773,8 @@
         <v>101</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21" s="20" t="s">
-        <v>103</v>
-      </c>
-      <c r="B21" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="C21" s="21">
-        <v>3</v>
-      </c>
-      <c r="D21" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="E21" s="22" t="s">
-        <v>105</v>
-      </c>
-      <c r="F21" s="22" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" ht="12.75" x14ac:dyDescent="0.2"/>
+    <row r="22" spans="1:6" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A22" s="20"/>
       <c r="B22" s="23"/>
       <c r="C22" s="23"/>
@@ -2816,6 +2844,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2901,15 +2930,15 @@
       <c r="A7" s="8">
         <v>0.42708333333333331</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="26" t="s">
         <v>115</v>
       </c>
       <c r="C7" s="4"/>
-      <c r="D7" s="25" t="s">
+      <c r="D7" s="26" t="s">
         <v>115</v>
       </c>
       <c r="E7" s="4"/>
-      <c r="F7" s="25" t="s">
+      <c r="F7" s="26" t="s">
         <v>115</v>
       </c>
     </row>
@@ -2917,31 +2946,31 @@
       <c r="A8" s="8">
         <v>0.4375</v>
       </c>
-      <c r="B8" s="26"/>
+      <c r="B8" s="31"/>
       <c r="C8" s="4"/>
-      <c r="D8" s="26"/>
+      <c r="D8" s="31"/>
       <c r="E8" s="4"/>
-      <c r="F8" s="26"/>
+      <c r="F8" s="31"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="8">
         <v>0.44791666666666669</v>
       </c>
-      <c r="B9" s="26"/>
+      <c r="B9" s="31"/>
       <c r="C9" s="4"/>
-      <c r="D9" s="26"/>
+      <c r="D9" s="31"/>
       <c r="E9" s="4"/>
-      <c r="F9" s="26"/>
+      <c r="F9" s="31"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="8">
         <v>0.45833333333333331</v>
       </c>
-      <c r="B10" s="26"/>
+      <c r="B10" s="31"/>
       <c r="C10" s="4"/>
-      <c r="D10" s="26"/>
+      <c r="D10" s="31"/>
       <c r="E10" s="4"/>
-      <c r="F10" s="26"/>
+      <c r="F10" s="31"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="8">
@@ -3057,15 +3086,15 @@
       <c r="A22" s="8">
         <v>0.58333333333333337</v>
       </c>
-      <c r="B22" s="25" t="s">
+      <c r="B22" s="26" t="s">
         <v>116</v>
       </c>
       <c r="C22" s="4"/>
-      <c r="D22" s="25" t="s">
+      <c r="D22" s="26" t="s">
         <v>116</v>
       </c>
       <c r="E22" s="4"/>
-      <c r="F22" s="25" t="s">
+      <c r="F22" s="26" t="s">
         <v>116</v>
       </c>
     </row>
@@ -3073,31 +3102,31 @@
       <c r="A23" s="8">
         <v>0.59375</v>
       </c>
-      <c r="B23" s="26"/>
+      <c r="B23" s="31"/>
       <c r="C23" s="4"/>
-      <c r="D23" s="26"/>
+      <c r="D23" s="31"/>
       <c r="E23" s="4"/>
-      <c r="F23" s="26"/>
+      <c r="F23" s="31"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="8">
         <v>0.60416666666666663</v>
       </c>
-      <c r="B24" s="26"/>
+      <c r="B24" s="31"/>
       <c r="C24" s="4"/>
-      <c r="D24" s="26"/>
+      <c r="D24" s="31"/>
       <c r="E24" s="4"/>
-      <c r="F24" s="26"/>
+      <c r="F24" s="31"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="8">
         <v>0.61458333333333337</v>
       </c>
-      <c r="B25" s="26"/>
+      <c r="B25" s="31"/>
       <c r="C25" s="4"/>
-      <c r="D25" s="26"/>
+      <c r="D25" s="31"/>
       <c r="E25" s="4"/>
-      <c r="F25" s="26"/>
+      <c r="F25" s="31"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="8">
@@ -3115,15 +3144,15 @@
       <c r="A27" s="8">
         <v>0.63541666666666663</v>
       </c>
-      <c r="B27" s="27" t="s">
+      <c r="B27" s="30" t="s">
         <v>117</v>
       </c>
       <c r="C27" s="6"/>
-      <c r="D27" s="27" t="s">
+      <c r="D27" s="30" t="s">
         <v>117</v>
       </c>
       <c r="E27" s="6"/>
-      <c r="F27" s="27" t="s">
+      <c r="F27" s="30" t="s">
         <v>117</v>
       </c>
     </row>
@@ -3131,31 +3160,31 @@
       <c r="A28" s="8">
         <v>0.64583333333333337</v>
       </c>
-      <c r="B28" s="26"/>
+      <c r="B28" s="31"/>
       <c r="C28" s="6"/>
-      <c r="D28" s="26"/>
+      <c r="D28" s="31"/>
       <c r="E28" s="6"/>
-      <c r="F28" s="26"/>
+      <c r="F28" s="31"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="8">
         <v>0.65625</v>
       </c>
-      <c r="B29" s="26"/>
+      <c r="B29" s="31"/>
       <c r="C29" s="6"/>
-      <c r="D29" s="26"/>
+      <c r="D29" s="31"/>
       <c r="E29" s="6"/>
-      <c r="F29" s="26"/>
+      <c r="F29" s="31"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="8">
         <v>0.66666666666666663</v>
       </c>
-      <c r="B30" s="26"/>
+      <c r="B30" s="31"/>
       <c r="C30" s="6"/>
-      <c r="D30" s="26"/>
+      <c r="D30" s="31"/>
       <c r="E30" s="6"/>
-      <c r="F30" s="26"/>
+      <c r="F30" s="31"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="8">

</xml_diff>